<commit_message>
Auto commit - 2025-02-25
</commit_message>
<xml_diff>
--- a/2024/2024_06_07_CB_loans/2_Money_Base_dayly_2025.xlsx
+++ b/2024/2024_06_07_CB_loans/2_Money_Base_dayly_2025.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54E8607B-9435-41D0-8B6E-0C2B316709ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="605"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="605" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name=" Eng actual exchange rate" sheetId="4" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -18,8 +19,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -27,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="66">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -240,11 +239,32 @@
   <si>
     <t>07.02.25</t>
   </si>
+  <si>
+    <t>10.02.25</t>
+  </si>
+  <si>
+    <t>11.02.25</t>
+  </si>
+  <si>
+    <t>12.02.25</t>
+  </si>
+  <si>
+    <t>13.02.25</t>
+  </si>
+  <si>
+    <t>14.02.25</t>
+  </si>
+  <si>
+    <t>17.02.25</t>
+  </si>
+  <si>
+    <t>18.02.25</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="6">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
@@ -1062,128 +1082,128 @@
     <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="121" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="122">
-    <cellStyle name=" Verticals" xfId="1"/>
-    <cellStyle name="_1_²ÜºÈÆø" xfId="2"/>
+    <cellStyle name=" Verticals" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="_1_²ÜºÈÆø" xfId="2" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="20% - Accent1" xfId="3" builtinId="30"/>
-    <cellStyle name="20% - Accent1 2" xfId="4"/>
-    <cellStyle name="20% - Accent2 2" xfId="5"/>
-    <cellStyle name="20% - Accent3 2" xfId="6"/>
-    <cellStyle name="20% - Accent4 2" xfId="7"/>
-    <cellStyle name="20% - Accent5 2" xfId="8"/>
-    <cellStyle name="20% - Accent6 2" xfId="9"/>
-    <cellStyle name="40% - Accent1 2" xfId="10"/>
-    <cellStyle name="40% - Accent2 2" xfId="11"/>
-    <cellStyle name="40% - Accent3 2" xfId="12"/>
-    <cellStyle name="40% - Accent4 2" xfId="13"/>
-    <cellStyle name="40% - Accent5 2" xfId="14"/>
-    <cellStyle name="40% - Accent6 2" xfId="15"/>
+    <cellStyle name="20% - Accent1 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="20% - Accent2 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="20% - Accent3 2" xfId="6" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="20% - Accent4 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="20% - Accent5 2" xfId="8" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="20% - Accent6 2" xfId="9" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
+    <cellStyle name="40% - Accent1 2" xfId="10" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
+    <cellStyle name="40% - Accent2 2" xfId="11" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
+    <cellStyle name="40% - Accent3 2" xfId="12" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
+    <cellStyle name="40% - Accent4 2" xfId="13" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
+    <cellStyle name="40% - Accent5 2" xfId="14" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
+    <cellStyle name="40% - Accent6 2" xfId="15" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
     <cellStyle name="60% - Accent1" xfId="16" builtinId="32"/>
-    <cellStyle name="60% - Accent1 2" xfId="17"/>
-    <cellStyle name="60% - Accent2 2" xfId="18"/>
-    <cellStyle name="60% - Accent3 2" xfId="19"/>
-    <cellStyle name="60% - Accent4 2" xfId="20"/>
-    <cellStyle name="60% - Accent5 2" xfId="21"/>
-    <cellStyle name="60% - Accent6 2" xfId="22"/>
-    <cellStyle name="Accent1 - 20%" xfId="23"/>
-    <cellStyle name="Accent1 - 40%" xfId="24"/>
-    <cellStyle name="Accent1 - 60%" xfId="25"/>
-    <cellStyle name="Accent1 2" xfId="26"/>
-    <cellStyle name="Accent2 - 20%" xfId="27"/>
-    <cellStyle name="Accent2 - 40%" xfId="28"/>
-    <cellStyle name="Accent2 - 60%" xfId="29"/>
-    <cellStyle name="Accent2 2" xfId="30"/>
-    <cellStyle name="Accent3 - 20%" xfId="31"/>
-    <cellStyle name="Accent3 - 40%" xfId="32"/>
-    <cellStyle name="Accent3 - 60%" xfId="33"/>
-    <cellStyle name="Accent3 2" xfId="34"/>
-    <cellStyle name="Accent4 - 20%" xfId="35"/>
-    <cellStyle name="Accent4 - 40%" xfId="36"/>
-    <cellStyle name="Accent4 - 60%" xfId="37"/>
-    <cellStyle name="Accent4 2" xfId="38"/>
-    <cellStyle name="Accent5 - 20%" xfId="39"/>
-    <cellStyle name="Accent5 - 40%" xfId="40"/>
-    <cellStyle name="Accent5 - 60%" xfId="41"/>
-    <cellStyle name="Accent5 2" xfId="42"/>
-    <cellStyle name="Accent6 - 20%" xfId="43"/>
-    <cellStyle name="Accent6 - 40%" xfId="44"/>
-    <cellStyle name="Accent6 - 60%" xfId="45"/>
-    <cellStyle name="Accent6 2" xfId="46"/>
-    <cellStyle name="al_laroux_7_laroux_1_²ðò²Ê´²ÜÎ" xfId="47"/>
-    <cellStyle name="Bad 2" xfId="48"/>
-    <cellStyle name="Body" xfId="49"/>
-    <cellStyle name="Calculation 2" xfId="50"/>
-    <cellStyle name="Check Cell 2" xfId="51"/>
+    <cellStyle name="60% - Accent1 2" xfId="17" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
+    <cellStyle name="60% - Accent2 2" xfId="18" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
+    <cellStyle name="60% - Accent3 2" xfId="19" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
+    <cellStyle name="60% - Accent4 2" xfId="20" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
+    <cellStyle name="60% - Accent5 2" xfId="21" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
+    <cellStyle name="60% - Accent6 2" xfId="22" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
+    <cellStyle name="Accent1 - 20%" xfId="23" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
+    <cellStyle name="Accent1 - 40%" xfId="24" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
+    <cellStyle name="Accent1 - 60%" xfId="25" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
+    <cellStyle name="Accent1 2" xfId="26" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
+    <cellStyle name="Accent2 - 20%" xfId="27" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
+    <cellStyle name="Accent2 - 40%" xfId="28" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
+    <cellStyle name="Accent2 - 60%" xfId="29" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
+    <cellStyle name="Accent2 2" xfId="30" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
+    <cellStyle name="Accent3 - 20%" xfId="31" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
+    <cellStyle name="Accent3 - 40%" xfId="32" xr:uid="{00000000-0005-0000-0000-00001F000000}"/>
+    <cellStyle name="Accent3 - 60%" xfId="33" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
+    <cellStyle name="Accent3 2" xfId="34" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
+    <cellStyle name="Accent4 - 20%" xfId="35" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
+    <cellStyle name="Accent4 - 40%" xfId="36" xr:uid="{00000000-0005-0000-0000-000023000000}"/>
+    <cellStyle name="Accent4 - 60%" xfId="37" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
+    <cellStyle name="Accent4 2" xfId="38" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
+    <cellStyle name="Accent5 - 20%" xfId="39" xr:uid="{00000000-0005-0000-0000-000026000000}"/>
+    <cellStyle name="Accent5 - 40%" xfId="40" xr:uid="{00000000-0005-0000-0000-000027000000}"/>
+    <cellStyle name="Accent5 - 60%" xfId="41" xr:uid="{00000000-0005-0000-0000-000028000000}"/>
+    <cellStyle name="Accent5 2" xfId="42" xr:uid="{00000000-0005-0000-0000-000029000000}"/>
+    <cellStyle name="Accent6 - 20%" xfId="43" xr:uid="{00000000-0005-0000-0000-00002A000000}"/>
+    <cellStyle name="Accent6 - 40%" xfId="44" xr:uid="{00000000-0005-0000-0000-00002B000000}"/>
+    <cellStyle name="Accent6 - 60%" xfId="45" xr:uid="{00000000-0005-0000-0000-00002C000000}"/>
+    <cellStyle name="Accent6 2" xfId="46" xr:uid="{00000000-0005-0000-0000-00002D000000}"/>
+    <cellStyle name="al_laroux_7_laroux_1_²ðò²Ê´²ÜÎ" xfId="47" xr:uid="{00000000-0005-0000-0000-00002E000000}"/>
+    <cellStyle name="Bad 2" xfId="48" xr:uid="{00000000-0005-0000-0000-00002F000000}"/>
+    <cellStyle name="Body" xfId="49" xr:uid="{00000000-0005-0000-0000-000030000000}"/>
+    <cellStyle name="Calculation 2" xfId="50" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
+    <cellStyle name="Check Cell 2" xfId="51" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
     <cellStyle name="Comma" xfId="52" builtinId="3"/>
-    <cellStyle name="Comma 2" xfId="53"/>
-    <cellStyle name="Comma 3" xfId="54"/>
-    <cellStyle name="Dezimal [0]_laroux" xfId="55"/>
-    <cellStyle name="Dezimal_laroux" xfId="56"/>
-    <cellStyle name="Emphasis 1" xfId="57"/>
-    <cellStyle name="Emphasis 2" xfId="58"/>
-    <cellStyle name="Emphasis 3" xfId="59"/>
-    <cellStyle name="Euro" xfId="60"/>
-    <cellStyle name="Explanatory Text 2" xfId="61"/>
-    <cellStyle name="Good 2" xfId="62"/>
-    <cellStyle name="Heading 1 2" xfId="63"/>
-    <cellStyle name="Heading 2 2" xfId="64"/>
-    <cellStyle name="Heading 3 2" xfId="65"/>
-    <cellStyle name="Heading 4 2" xfId="66"/>
+    <cellStyle name="Comma 2" xfId="53" xr:uid="{00000000-0005-0000-0000-000034000000}"/>
+    <cellStyle name="Comma 3" xfId="54" xr:uid="{00000000-0005-0000-0000-000035000000}"/>
+    <cellStyle name="Dezimal [0]_laroux" xfId="55" xr:uid="{00000000-0005-0000-0000-000036000000}"/>
+    <cellStyle name="Dezimal_laroux" xfId="56" xr:uid="{00000000-0005-0000-0000-000037000000}"/>
+    <cellStyle name="Emphasis 1" xfId="57" xr:uid="{00000000-0005-0000-0000-000038000000}"/>
+    <cellStyle name="Emphasis 2" xfId="58" xr:uid="{00000000-0005-0000-0000-000039000000}"/>
+    <cellStyle name="Emphasis 3" xfId="59" xr:uid="{00000000-0005-0000-0000-00003A000000}"/>
+    <cellStyle name="Euro" xfId="60" xr:uid="{00000000-0005-0000-0000-00003B000000}"/>
+    <cellStyle name="Explanatory Text 2" xfId="61" xr:uid="{00000000-0005-0000-0000-00003C000000}"/>
+    <cellStyle name="Good 2" xfId="62" xr:uid="{00000000-0005-0000-0000-00003D000000}"/>
+    <cellStyle name="Heading 1 2" xfId="63" xr:uid="{00000000-0005-0000-0000-00003E000000}"/>
+    <cellStyle name="Heading 2 2" xfId="64" xr:uid="{00000000-0005-0000-0000-00003F000000}"/>
+    <cellStyle name="Heading 3 2" xfId="65" xr:uid="{00000000-0005-0000-0000-000040000000}"/>
+    <cellStyle name="Heading 4 2" xfId="66" xr:uid="{00000000-0005-0000-0000-000041000000}"/>
     <cellStyle name="Hyperlink" xfId="121" builtinId="8"/>
-    <cellStyle name="Îáû÷íûé_AMD" xfId="67"/>
-    <cellStyle name="Input 2" xfId="68"/>
-    <cellStyle name="Linked Cell 2" xfId="69"/>
-    <cellStyle name="Milliers [0]_laroux" xfId="70"/>
-    <cellStyle name="Milliers_laroux" xfId="71"/>
-    <cellStyle name="Neutral 2" xfId="72"/>
-    <cellStyle name="no dec" xfId="73"/>
+    <cellStyle name="Îáû÷íûé_AMD" xfId="67" xr:uid="{00000000-0005-0000-0000-000043000000}"/>
+    <cellStyle name="Input 2" xfId="68" xr:uid="{00000000-0005-0000-0000-000044000000}"/>
+    <cellStyle name="Linked Cell 2" xfId="69" xr:uid="{00000000-0005-0000-0000-000045000000}"/>
+    <cellStyle name="Milliers [0]_laroux" xfId="70" xr:uid="{00000000-0005-0000-0000-000046000000}"/>
+    <cellStyle name="Milliers_laroux" xfId="71" xr:uid="{00000000-0005-0000-0000-000047000000}"/>
+    <cellStyle name="Neutral 2" xfId="72" xr:uid="{00000000-0005-0000-0000-000048000000}"/>
+    <cellStyle name="no dec" xfId="73" xr:uid="{00000000-0005-0000-0000-000049000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal - Style1" xfId="74"/>
-    <cellStyle name="Normal 10" xfId="75"/>
-    <cellStyle name="Normal 10 2" xfId="76"/>
-    <cellStyle name="Normal 11" xfId="77"/>
-    <cellStyle name="Normal 11 2" xfId="78"/>
-    <cellStyle name="Normal 12" xfId="79"/>
-    <cellStyle name="Normal 12 2" xfId="80"/>
-    <cellStyle name="Normal 13" xfId="81"/>
-    <cellStyle name="Normal 13 2" xfId="82"/>
-    <cellStyle name="Normal 14" xfId="83"/>
-    <cellStyle name="Normal 14 2" xfId="84"/>
-    <cellStyle name="Normal 16" xfId="85"/>
-    <cellStyle name="Normal 17" xfId="86"/>
-    <cellStyle name="Normal 18" xfId="87"/>
-    <cellStyle name="Normal 19" xfId="88"/>
-    <cellStyle name="Normal 2 10" xfId="89"/>
-    <cellStyle name="Normal 2 11" xfId="90"/>
-    <cellStyle name="Normal 2 2" xfId="91"/>
-    <cellStyle name="Normal 2 3" xfId="92"/>
-    <cellStyle name="Normal 2 4" xfId="93"/>
-    <cellStyle name="Normal 2 5" xfId="94"/>
-    <cellStyle name="Normal 2 6" xfId="95"/>
-    <cellStyle name="Normal 2 7" xfId="96"/>
-    <cellStyle name="Normal 2 8" xfId="97"/>
-    <cellStyle name="Normal 2 9" xfId="98"/>
-    <cellStyle name="Normal 20" xfId="99"/>
-    <cellStyle name="Normal 21" xfId="100"/>
-    <cellStyle name="Normal 22" xfId="101"/>
-    <cellStyle name="Normal 23" xfId="102"/>
-    <cellStyle name="Normal 3 2" xfId="103"/>
-    <cellStyle name="Normal 5 2" xfId="104"/>
-    <cellStyle name="Normal 6 2" xfId="105"/>
-    <cellStyle name="Normal 7 2" xfId="106"/>
-    <cellStyle name="Note 2" xfId="107"/>
-    <cellStyle name="Output 2" xfId="108"/>
-    <cellStyle name="Percent 2" xfId="109"/>
-    <cellStyle name="Percent 3" xfId="110"/>
-    <cellStyle name="Sheet Title" xfId="111"/>
-    <cellStyle name="Standard_laroux" xfId="112"/>
-    <cellStyle name="Style 1" xfId="113"/>
-    <cellStyle name="Style 2" xfId="114"/>
-    <cellStyle name="Title 2" xfId="115"/>
-    <cellStyle name="Total 2" xfId="116"/>
-    <cellStyle name="ux" xfId="117"/>
-    <cellStyle name="Währung [0]_laroux" xfId="118"/>
-    <cellStyle name="Währung_laroux" xfId="119"/>
-    <cellStyle name="Warning Text 2" xfId="120"/>
+    <cellStyle name="Normal - Style1" xfId="74" xr:uid="{00000000-0005-0000-0000-00004B000000}"/>
+    <cellStyle name="Normal 10" xfId="75" xr:uid="{00000000-0005-0000-0000-00004C000000}"/>
+    <cellStyle name="Normal 10 2" xfId="76" xr:uid="{00000000-0005-0000-0000-00004D000000}"/>
+    <cellStyle name="Normal 11" xfId="77" xr:uid="{00000000-0005-0000-0000-00004E000000}"/>
+    <cellStyle name="Normal 11 2" xfId="78" xr:uid="{00000000-0005-0000-0000-00004F000000}"/>
+    <cellStyle name="Normal 12" xfId="79" xr:uid="{00000000-0005-0000-0000-000050000000}"/>
+    <cellStyle name="Normal 12 2" xfId="80" xr:uid="{00000000-0005-0000-0000-000051000000}"/>
+    <cellStyle name="Normal 13" xfId="81" xr:uid="{00000000-0005-0000-0000-000052000000}"/>
+    <cellStyle name="Normal 13 2" xfId="82" xr:uid="{00000000-0005-0000-0000-000053000000}"/>
+    <cellStyle name="Normal 14" xfId="83" xr:uid="{00000000-0005-0000-0000-000054000000}"/>
+    <cellStyle name="Normal 14 2" xfId="84" xr:uid="{00000000-0005-0000-0000-000055000000}"/>
+    <cellStyle name="Normal 16" xfId="85" xr:uid="{00000000-0005-0000-0000-000056000000}"/>
+    <cellStyle name="Normal 17" xfId="86" xr:uid="{00000000-0005-0000-0000-000057000000}"/>
+    <cellStyle name="Normal 18" xfId="87" xr:uid="{00000000-0005-0000-0000-000058000000}"/>
+    <cellStyle name="Normal 19" xfId="88" xr:uid="{00000000-0005-0000-0000-000059000000}"/>
+    <cellStyle name="Normal 2 10" xfId="89" xr:uid="{00000000-0005-0000-0000-00005A000000}"/>
+    <cellStyle name="Normal 2 11" xfId="90" xr:uid="{00000000-0005-0000-0000-00005B000000}"/>
+    <cellStyle name="Normal 2 2" xfId="91" xr:uid="{00000000-0005-0000-0000-00005C000000}"/>
+    <cellStyle name="Normal 2 3" xfId="92" xr:uid="{00000000-0005-0000-0000-00005D000000}"/>
+    <cellStyle name="Normal 2 4" xfId="93" xr:uid="{00000000-0005-0000-0000-00005E000000}"/>
+    <cellStyle name="Normal 2 5" xfId="94" xr:uid="{00000000-0005-0000-0000-00005F000000}"/>
+    <cellStyle name="Normal 2 6" xfId="95" xr:uid="{00000000-0005-0000-0000-000060000000}"/>
+    <cellStyle name="Normal 2 7" xfId="96" xr:uid="{00000000-0005-0000-0000-000061000000}"/>
+    <cellStyle name="Normal 2 8" xfId="97" xr:uid="{00000000-0005-0000-0000-000062000000}"/>
+    <cellStyle name="Normal 2 9" xfId="98" xr:uid="{00000000-0005-0000-0000-000063000000}"/>
+    <cellStyle name="Normal 20" xfId="99" xr:uid="{00000000-0005-0000-0000-000064000000}"/>
+    <cellStyle name="Normal 21" xfId="100" xr:uid="{00000000-0005-0000-0000-000065000000}"/>
+    <cellStyle name="Normal 22" xfId="101" xr:uid="{00000000-0005-0000-0000-000066000000}"/>
+    <cellStyle name="Normal 23" xfId="102" xr:uid="{00000000-0005-0000-0000-000067000000}"/>
+    <cellStyle name="Normal 3 2" xfId="103" xr:uid="{00000000-0005-0000-0000-000068000000}"/>
+    <cellStyle name="Normal 5 2" xfId="104" xr:uid="{00000000-0005-0000-0000-000069000000}"/>
+    <cellStyle name="Normal 6 2" xfId="105" xr:uid="{00000000-0005-0000-0000-00006A000000}"/>
+    <cellStyle name="Normal 7 2" xfId="106" xr:uid="{00000000-0005-0000-0000-00006B000000}"/>
+    <cellStyle name="Note 2" xfId="107" xr:uid="{00000000-0005-0000-0000-00006C000000}"/>
+    <cellStyle name="Output 2" xfId="108" xr:uid="{00000000-0005-0000-0000-00006D000000}"/>
+    <cellStyle name="Percent 2" xfId="109" xr:uid="{00000000-0005-0000-0000-00006E000000}"/>
+    <cellStyle name="Percent 3" xfId="110" xr:uid="{00000000-0005-0000-0000-00006F000000}"/>
+    <cellStyle name="Sheet Title" xfId="111" xr:uid="{00000000-0005-0000-0000-000070000000}"/>
+    <cellStyle name="Standard_laroux" xfId="112" xr:uid="{00000000-0005-0000-0000-000071000000}"/>
+    <cellStyle name="Style 1" xfId="113" xr:uid="{00000000-0005-0000-0000-000072000000}"/>
+    <cellStyle name="Style 2" xfId="114" xr:uid="{00000000-0005-0000-0000-000073000000}"/>
+    <cellStyle name="Title 2" xfId="115" xr:uid="{00000000-0005-0000-0000-000074000000}"/>
+    <cellStyle name="Total 2" xfId="116" xr:uid="{00000000-0005-0000-0000-000075000000}"/>
+    <cellStyle name="ux" xfId="117" xr:uid="{00000000-0005-0000-0000-000076000000}"/>
+    <cellStyle name="Währung [0]_laroux" xfId="118" xr:uid="{00000000-0005-0000-0000-000077000000}"/>
+    <cellStyle name="Währung_laroux" xfId="119" xr:uid="{00000000-0005-0000-0000-000078000000}"/>
+    <cellStyle name="Warning Text 2" xfId="120" xr:uid="{00000000-0005-0000-0000-000079000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1342,6 +1362,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -1377,6 +1414,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1552,38 +1606,38 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AL63"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AS63"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="15.6" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="55.140625" style="18" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="55.109375" style="18" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" style="7" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" style="7" customWidth="1"/>
     <col min="4" max="4" width="16" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" style="7" bestFit="1" customWidth="1"/>
     <col min="6" max="14" width="16" style="7" bestFit="1" customWidth="1"/>
     <col min="15" max="32" width="16" style="7" hidden="1" customWidth="1"/>
-    <col min="33" max="38" width="16" style="7" bestFit="1" customWidth="1"/>
-    <col min="39" max="16384" width="11.5703125" style="7"/>
+    <col min="33" max="45" width="16" style="7" bestFit="1" customWidth="1"/>
+    <col min="46" max="16384" width="11.5546875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" s="24" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:45" s="24" customFormat="1" ht="15" x14ac:dyDescent="0.35">
       <c r="A1" s="23" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:38" s="24" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:45" s="24" customFormat="1" ht="15" x14ac:dyDescent="0.35">
       <c r="A2" s="23" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:38" ht="7.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:45" ht="7.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8"/>
     </row>
-    <row r="4" spans="1:38" ht="3" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:45" ht="3" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="9"/>
     </row>
-    <row r="5" spans="1:38" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:45" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -1698,8 +1752,29 @@
       <c r="AL5" s="10" t="s">
         <v>58</v>
       </c>
+      <c r="AM5" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="AN5" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="AO5" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="AP5" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="AQ5" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="AR5" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="AS5" s="10" t="s">
+        <v>65</v>
+      </c>
     </row>
-    <row r="6" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A6" s="11"/>
       <c r="B6" s="12"/>
       <c r="C6" s="12"/>
@@ -1738,8 +1813,15 @@
       <c r="AJ6" s="12"/>
       <c r="AK6" s="12"/>
       <c r="AL6" s="12"/>
+      <c r="AM6" s="12"/>
+      <c r="AN6" s="12"/>
+      <c r="AO6" s="12"/>
+      <c r="AP6" s="12"/>
+      <c r="AQ6" s="12"/>
+      <c r="AR6" s="12"/>
+      <c r="AS6" s="12"/>
     </row>
-    <row r="7" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>26</v>
       </c>
@@ -1854,8 +1936,29 @@
       <c r="AL7" s="13">
         <v>1032757.912501425</v>
       </c>
+      <c r="AM7" s="13">
+        <v>1028079.2500539343</v>
+      </c>
+      <c r="AN7" s="13">
+        <v>1035440.4419206465</v>
+      </c>
+      <c r="AO7" s="13">
+        <v>1044491.1513781439</v>
+      </c>
+      <c r="AP7" s="13">
+        <v>1055248.7584258004</v>
+      </c>
+      <c r="AQ7" s="13">
+        <v>1047909.7364307392</v>
+      </c>
+      <c r="AR7" s="13">
+        <v>1043546.8312335956</v>
+      </c>
+      <c r="AS7" s="13">
+        <v>1005841.1497386224</v>
+      </c>
     </row>
-    <row r="8" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -1970,8 +2073,29 @@
       <c r="AL8" s="13">
         <v>759008.84884377499</v>
       </c>
+      <c r="AM8" s="13">
+        <v>755214.61249436578</v>
+      </c>
+      <c r="AN8" s="13">
+        <v>727168.63653615373</v>
+      </c>
+      <c r="AO8" s="13">
+        <v>741625.50244545599</v>
+      </c>
+      <c r="AP8" s="13">
+        <v>751016.61052999971</v>
+      </c>
+      <c r="AQ8" s="13">
+        <v>756777.14395006059</v>
+      </c>
+      <c r="AR8" s="13">
+        <v>764023.44775720418</v>
+      </c>
+      <c r="AS8" s="13">
+        <v>779391.73407917749</v>
+      </c>
     </row>
-    <row r="9" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -2086,8 +2210,29 @@
       <c r="AL9" s="13">
         <v>-510667.29164730001</v>
       </c>
+      <c r="AM9" s="13">
+        <v>-510423.01821410004</v>
+      </c>
+      <c r="AN9" s="13">
+        <v>-509578.36385540001</v>
+      </c>
+      <c r="AO9" s="13">
+        <v>-547625.21648910001</v>
+      </c>
+      <c r="AP9" s="13">
+        <v>-538825.83877859986</v>
+      </c>
+      <c r="AQ9" s="13">
+        <v>-534200.94945959991</v>
+      </c>
+      <c r="AR9" s="13">
+        <v>-527196.57984949986</v>
+      </c>
+      <c r="AS9" s="13">
+        <v>-512049.90239390009</v>
+      </c>
     </row>
-    <row r="10" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>3</v>
       </c>
@@ -2202,8 +2347,29 @@
       <c r="AL10" s="13">
         <v>854600.90225029993</v>
       </c>
+      <c r="AM10" s="13">
+        <v>848117.98492229998</v>
+      </c>
+      <c r="AN10" s="13">
+        <v>821759.49847410002</v>
+      </c>
+      <c r="AO10" s="13">
+        <v>851885.04499890003</v>
+      </c>
+      <c r="AP10" s="13">
+        <v>852043.7714472001</v>
+      </c>
+      <c r="AQ10" s="13">
+        <v>854526.7015503</v>
+      </c>
+      <c r="AR10" s="13">
+        <v>854997.16260119993</v>
+      </c>
+      <c r="AS10" s="13">
+        <v>855251.53183199989</v>
+      </c>
     </row>
-    <row r="11" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>17</v>
       </c>
@@ -2318,8 +2484,29 @@
       <c r="AL11" s="13">
         <v>545209.89078400005</v>
       </c>
+      <c r="AM11" s="13">
+        <v>545524.72696100001</v>
+      </c>
+      <c r="AN11" s="13">
+        <v>545629.67235000001</v>
+      </c>
+      <c r="AO11" s="13">
+        <v>560000</v>
+      </c>
+      <c r="AP11" s="13">
+        <v>560107.60934800003</v>
+      </c>
+      <c r="AQ11" s="13">
+        <v>560215.21870000008</v>
+      </c>
+      <c r="AR11" s="13">
+        <v>560538.04674800008</v>
+      </c>
+      <c r="AS11" s="13">
+        <v>560645.65609900001</v>
+      </c>
     </row>
-    <row r="12" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>22</v>
       </c>
@@ -2434,8 +2621,29 @@
       <c r="AL12" s="13">
         <v>545209.89078400005</v>
       </c>
+      <c r="AM12" s="13">
+        <v>545524.72696100001</v>
+      </c>
+      <c r="AN12" s="13">
+        <v>545629.67235000001</v>
+      </c>
+      <c r="AO12" s="13">
+        <v>560000</v>
+      </c>
+      <c r="AP12" s="13">
+        <v>560107.60934800003</v>
+      </c>
+      <c r="AQ12" s="13">
+        <v>560215.21869999997</v>
+      </c>
+      <c r="AR12" s="13">
+        <v>560538.04674799996</v>
+      </c>
+      <c r="AS12" s="13">
+        <v>560645.65609900001</v>
+      </c>
     </row>
-    <row r="13" spans="1:38" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:45" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -2550,8 +2758,29 @@
       <c r="AL13" s="13">
         <v>0</v>
       </c>
+      <c r="AM13" s="13">
+        <v>0</v>
+      </c>
+      <c r="AN13" s="13">
+        <v>0</v>
+      </c>
+      <c r="AO13" s="13">
+        <v>0</v>
+      </c>
+      <c r="AP13" s="13">
+        <v>0</v>
+      </c>
+      <c r="AQ13" s="13">
+        <v>0</v>
+      </c>
+      <c r="AR13" s="13">
+        <v>0</v>
+      </c>
+      <c r="AS13" s="13">
+        <v>0</v>
+      </c>
     </row>
-    <row r="14" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>24</v>
       </c>
@@ -2666,8 +2895,29 @@
       <c r="AL14" s="13">
         <v>0</v>
       </c>
+      <c r="AM14" s="13">
+        <v>0</v>
+      </c>
+      <c r="AN14" s="13">
+        <v>0</v>
+      </c>
+      <c r="AO14" s="13">
+        <v>0</v>
+      </c>
+      <c r="AP14" s="13">
+        <v>0</v>
+      </c>
+      <c r="AQ14" s="13">
+        <v>0</v>
+      </c>
+      <c r="AR14" s="13">
+        <v>0</v>
+      </c>
+      <c r="AS14" s="13">
+        <v>0</v>
+      </c>
     </row>
-    <row r="15" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>25</v>
       </c>
@@ -2782,8 +3032,29 @@
       <c r="AL15" s="13">
         <v>0</v>
       </c>
+      <c r="AM15" s="13">
+        <v>0</v>
+      </c>
+      <c r="AN15" s="13">
+        <v>0</v>
+      </c>
+      <c r="AO15" s="13">
+        <v>0</v>
+      </c>
+      <c r="AP15" s="13">
+        <v>0</v>
+      </c>
+      <c r="AQ15" s="13">
+        <v>0</v>
+      </c>
+      <c r="AR15" s="13">
+        <v>0</v>
+      </c>
+      <c r="AS15" s="13">
+        <v>0</v>
+      </c>
     </row>
-    <row r="16" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>9</v>
       </c>
@@ -2898,8 +3169,29 @@
       <c r="AL16" s="13">
         <v>0</v>
       </c>
+      <c r="AM16" s="13">
+        <v>0</v>
+      </c>
+      <c r="AN16" s="13">
+        <v>0</v>
+      </c>
+      <c r="AO16" s="13">
+        <v>0</v>
+      </c>
+      <c r="AP16" s="13">
+        <v>0</v>
+      </c>
+      <c r="AQ16" s="13">
+        <v>0</v>
+      </c>
+      <c r="AR16" s="13">
+        <v>0</v>
+      </c>
+      <c r="AS16" s="13">
+        <v>0</v>
+      </c>
     </row>
-    <row r="17" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>10</v>
       </c>
@@ -3014,8 +3306,27 @@
       <c r="AL17" s="13">
         <v>-3000.4315068000001</v>
       </c>
+      <c r="AM17" s="13">
+        <v>-9951.4311644000009</v>
+      </c>
+      <c r="AN17" s="13">
+        <v>-36455.242808200004</v>
+      </c>
+      <c r="AO17" s="13"/>
+      <c r="AP17" s="13">
+        <v>0</v>
+      </c>
+      <c r="AQ17" s="13">
+        <v>0</v>
+      </c>
+      <c r="AR17" s="13">
+        <v>0</v>
+      </c>
+      <c r="AS17" s="13">
+        <v>0</v>
+      </c>
     </row>
-    <row r="18" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>12</v>
       </c>
@@ -3130,8 +3441,29 @@
       <c r="AL18" s="13">
         <v>0</v>
       </c>
+      <c r="AM18" s="13">
+        <v>0</v>
+      </c>
+      <c r="AN18" s="13">
+        <v>0</v>
+      </c>
+      <c r="AO18" s="13">
+        <v>0</v>
+      </c>
+      <c r="AP18" s="13">
+        <v>0</v>
+      </c>
+      <c r="AQ18" s="13">
+        <v>0</v>
+      </c>
+      <c r="AR18" s="13">
+        <v>0</v>
+      </c>
+      <c r="AS18" s="13">
+        <v>0</v>
+      </c>
     </row>
-    <row r="19" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
@@ -3246,8 +3578,29 @@
       <c r="AL19" s="13">
         <v>0</v>
       </c>
+      <c r="AM19" s="13">
+        <v>0</v>
+      </c>
+      <c r="AN19" s="13">
+        <v>0</v>
+      </c>
+      <c r="AO19" s="13">
+        <v>0</v>
+      </c>
+      <c r="AP19" s="13">
+        <v>0</v>
+      </c>
+      <c r="AQ19" s="13">
+        <v>0</v>
+      </c>
+      <c r="AR19" s="13">
+        <v>0</v>
+      </c>
+      <c r="AS19" s="13">
+        <v>0</v>
+      </c>
     </row>
-    <row r="20" spans="1:38" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:45" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>11</v>
       </c>
@@ -3362,8 +3715,29 @@
       <c r="AL20" s="13">
         <v>0</v>
       </c>
+      <c r="AM20" s="13">
+        <v>0</v>
+      </c>
+      <c r="AN20" s="13">
+        <v>0</v>
+      </c>
+      <c r="AO20" s="13">
+        <v>0</v>
+      </c>
+      <c r="AP20" s="13">
+        <v>0</v>
+      </c>
+      <c r="AQ20" s="13">
+        <v>0</v>
+      </c>
+      <c r="AR20" s="13">
+        <v>0</v>
+      </c>
+      <c r="AS20" s="13">
+        <v>0</v>
+      </c>
     </row>
-    <row r="21" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>16</v>
       </c>
@@ -3478,8 +3852,29 @@
       <c r="AL21" s="13">
         <v>0</v>
       </c>
+      <c r="AM21" s="13">
+        <v>0</v>
+      </c>
+      <c r="AN21" s="13">
+        <v>0</v>
+      </c>
+      <c r="AO21" s="13">
+        <v>0</v>
+      </c>
+      <c r="AP21" s="13">
+        <v>0</v>
+      </c>
+      <c r="AQ21" s="13">
+        <v>0</v>
+      </c>
+      <c r="AR21" s="13">
+        <v>0</v>
+      </c>
+      <c r="AS21" s="13">
+        <v>0</v>
+      </c>
     </row>
-    <row r="22" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -3594,8 +3989,29 @@
       <c r="AL22" s="13">
         <v>415075.23824077495</v>
       </c>
+      <c r="AM22" s="13">
+        <v>417519.64578616584</v>
+      </c>
+      <c r="AN22" s="13">
+        <v>414987.5019174536</v>
+      </c>
+      <c r="AO22" s="13">
+        <v>437365.67393565597</v>
+      </c>
+      <c r="AP22" s="13">
+        <v>437798.67786139948</v>
+      </c>
+      <c r="AQ22" s="13">
+        <v>436451.3918593605</v>
+      </c>
+      <c r="AR22" s="13">
+        <v>436222.86500550411</v>
+      </c>
+      <c r="AS22" s="13">
+        <v>436190.10464107769</v>
+      </c>
     </row>
-    <row r="23" spans="1:38" s="21" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:45" s="21" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="19" t="s">
         <v>4</v>
       </c>
@@ -3710,8 +4126,29 @@
       <c r="AL23" s="20">
         <v>1791766.7613452</v>
       </c>
+      <c r="AM23" s="20">
+        <v>1783293.8625483001</v>
+      </c>
+      <c r="AN23" s="20">
+        <v>1762609.0784568002</v>
+      </c>
+      <c r="AO23" s="20">
+        <v>1786116.6538235999</v>
+      </c>
+      <c r="AP23" s="20">
+        <v>1806265.3689558001</v>
+      </c>
+      <c r="AQ23" s="20">
+        <v>1804686.8803807998</v>
+      </c>
+      <c r="AR23" s="20">
+        <v>1807570.2789907998</v>
+      </c>
+      <c r="AS23" s="20">
+        <v>1785232.8838177999</v>
+      </c>
     </row>
-    <row r="24" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>5</v>
       </c>
@@ -3826,8 +4263,29 @@
       <c r="AL24" s="13">
         <v>945542.41051940003</v>
       </c>
+      <c r="AM24" s="13">
+        <v>948788.66756859992</v>
+      </c>
+      <c r="AN24" s="13">
+        <v>949351.44643429993</v>
+      </c>
+      <c r="AO24" s="13">
+        <v>947175.55223429995</v>
+      </c>
+      <c r="AP24" s="13">
+        <v>947165.11236469995</v>
+      </c>
+      <c r="AQ24" s="13">
+        <v>950780.86551469995</v>
+      </c>
+      <c r="AR24" s="13">
+        <v>950002.67689560005</v>
+      </c>
+      <c r="AS24" s="13">
+        <v>948166.86852659995</v>
+      </c>
     </row>
-    <row r="25" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>14</v>
       </c>
@@ -3942,8 +4400,29 @@
       <c r="AL25" s="13">
         <v>377653.36221950001</v>
       </c>
+      <c r="AM25" s="13">
+        <v>372236.41535340005</v>
+      </c>
+      <c r="AN25" s="13">
+        <v>347003.8387733</v>
+      </c>
+      <c r="AO25" s="13">
+        <v>365578.06095020002</v>
+      </c>
+      <c r="AP25" s="13">
+        <v>376491.1911308</v>
+      </c>
+      <c r="AQ25" s="13">
+        <v>368814.139012</v>
+      </c>
+      <c r="AR25" s="13">
+        <v>368776.14568710001</v>
+      </c>
+      <c r="AS25" s="13">
+        <v>361501.80517359998</v>
+      </c>
     </row>
-    <row r="26" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>13</v>
       </c>
@@ -4058,8 +4537,29 @@
       <c r="AL26" s="13">
         <v>455139.19663040002</v>
       </c>
+      <c r="AM26" s="13">
+        <v>452577.3877507</v>
+      </c>
+      <c r="AN26" s="13">
+        <v>455298.48593530001</v>
+      </c>
+      <c r="AO26" s="13">
+        <v>462265.92327219999</v>
+      </c>
+      <c r="AP26" s="13">
+        <v>469366.72135740001</v>
+      </c>
+      <c r="AQ26" s="13">
+        <v>475672.49726309994</v>
+      </c>
+      <c r="AR26" s="13">
+        <v>472581.13777229999</v>
+      </c>
+      <c r="AS26" s="13">
+        <v>463803.01439809997</v>
+      </c>
     </row>
-    <row r="27" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
         <v>32</v>
       </c>
@@ -4156,8 +4656,29 @@
       <c r="AL27" s="13">
         <v>1.2793298</v>
       </c>
+      <c r="AM27" s="13">
+        <v>1.2793298</v>
+      </c>
+      <c r="AN27" s="13">
+        <v>1.2777507000000001</v>
+      </c>
+      <c r="AO27" s="13">
+        <v>1.2777507000000001</v>
+      </c>
+      <c r="AP27" s="13">
+        <v>1.2777507000000001</v>
+      </c>
+      <c r="AQ27" s="13">
+        <v>1.2777507000000001</v>
+      </c>
+      <c r="AR27" s="13">
+        <v>1.2777507000000001</v>
+      </c>
+      <c r="AS27" s="13">
+        <v>1.2516696999999999</v>
+      </c>
     </row>
-    <row r="28" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>33</v>
       </c>
@@ -4254,8 +4775,29 @@
       <c r="AL28" s="13">
         <v>710.91545539999993</v>
       </c>
+      <c r="AM28" s="13">
+        <v>446.81464549999998</v>
+      </c>
+      <c r="AN28" s="13">
+        <v>446.92077430000001</v>
+      </c>
+      <c r="AO28" s="13">
+        <v>447.41280819999997</v>
+      </c>
+      <c r="AP28" s="13">
+        <v>447.66203480000001</v>
+      </c>
+      <c r="AQ28" s="13">
+        <v>448.10484309999998</v>
+      </c>
+      <c r="AR28" s="13">
+        <v>448.10267920000001</v>
+      </c>
+      <c r="AS28" s="13">
+        <v>447.80432589999998</v>
+      </c>
     </row>
-    <row r="29" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>6</v>
       </c>
@@ -4370,8 +4912,29 @@
       <c r="AL29" s="13">
         <v>12719.597190699949</v>
       </c>
+      <c r="AM29" s="13">
+        <v>9243.2979003000928</v>
+      </c>
+      <c r="AN29" s="13">
+        <v>10507.108788900267</v>
+      </c>
+      <c r="AO29" s="13">
+        <v>10648.426807999969</v>
+      </c>
+      <c r="AP29" s="13">
+        <v>12793.404317400127</v>
+      </c>
+      <c r="AQ29" s="13">
+        <v>8969.9959971998705</v>
+      </c>
+      <c r="AR29" s="13">
+        <v>15760.938205899749</v>
+      </c>
+      <c r="AS29" s="13">
+        <v>11312.139723899956</v>
+      </c>
     </row>
-    <row r="30" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
         <v>7</v>
       </c>
@@ -4486,8 +5049,29 @@
       <c r="AL30" s="13">
         <v>8068.8463656000004</v>
       </c>
+      <c r="AM30" s="13">
+        <v>5699.3612529999991</v>
+      </c>
+      <c r="AN30" s="13">
+        <v>6133.0974717999998</v>
+      </c>
+      <c r="AO30" s="13">
+        <v>6261.4630039999993</v>
+      </c>
+      <c r="AP30" s="13">
+        <v>6250.4232988000003</v>
+      </c>
+      <c r="AQ30" s="13">
+        <v>5607.7414080999997</v>
+      </c>
+      <c r="AR30" s="13">
+        <v>7584.2812804999994</v>
+      </c>
+      <c r="AS30" s="13">
+        <v>7589.2591434000005</v>
+      </c>
     </row>
-    <row r="31" spans="1:38" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:45" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>8</v>
       </c>
@@ -4602,8 +5186,29 @@
       <c r="AL31" s="13">
         <v>4650.7508250999999</v>
       </c>
+      <c r="AM31" s="13">
+        <v>3543.9366473000005</v>
+      </c>
+      <c r="AN31" s="13">
+        <v>4374.0113171000003</v>
+      </c>
+      <c r="AO31" s="13">
+        <v>4386.963804</v>
+      </c>
+      <c r="AP31" s="13">
+        <v>6542.9810186000004</v>
+      </c>
+      <c r="AQ31" s="13">
+        <v>3362.2545891</v>
+      </c>
+      <c r="AR31" s="13">
+        <v>8176.6569253999996</v>
+      </c>
+      <c r="AS31" s="13">
+        <v>3722.8805805000002</v>
+      </c>
     </row>
-    <row r="32" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A32" s="2"/>
       <c r="B32" s="14"/>
       <c r="C32" s="14"/>
@@ -4642,8 +5247,15 @@
       <c r="AJ32" s="14"/>
       <c r="AK32" s="14"/>
       <c r="AL32" s="14"/>
+      <c r="AM32" s="14"/>
+      <c r="AN32" s="14"/>
+      <c r="AO32" s="14"/>
+      <c r="AP32" s="14"/>
+      <c r="AQ32" s="14"/>
+      <c r="AR32" s="14"/>
+      <c r="AS32" s="14"/>
     </row>
-    <row r="33" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A33" s="6" t="s">
         <v>15</v>
       </c>
@@ -4684,8 +5296,15 @@
       <c r="AJ33" s="15"/>
       <c r="AK33" s="15"/>
       <c r="AL33" s="15"/>
+      <c r="AM33" s="15"/>
+      <c r="AN33" s="15"/>
+      <c r="AO33" s="15"/>
+      <c r="AP33" s="15"/>
+      <c r="AQ33" s="15"/>
+      <c r="AR33" s="15"/>
+      <c r="AS33" s="15"/>
     </row>
-    <row r="34" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A34" s="2"/>
       <c r="B34" s="16"/>
       <c r="C34" s="16"/>
@@ -4724,8 +5343,15 @@
       <c r="AJ34" s="16"/>
       <c r="AK34" s="16"/>
       <c r="AL34" s="16"/>
+      <c r="AM34" s="16"/>
+      <c r="AN34" s="16"/>
+      <c r="AO34" s="16"/>
+      <c r="AP34" s="16"/>
+      <c r="AQ34" s="16"/>
+      <c r="AR34" s="16"/>
+      <c r="AS34" s="16"/>
     </row>
-    <row r="35" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>26</v>
       </c>
@@ -4735,7 +5361,7 @@
         <v>-10609.381967150373</v>
       </c>
       <c r="D35" s="14">
-        <f t="shared" ref="D35:AL35" si="1">D7-C7</f>
+        <f t="shared" ref="D35:AS35" si="1">D7-C7</f>
         <v>-76669.83926140063</v>
       </c>
       <c r="E35" s="14">
@@ -4874,8 +5500,36 @@
         <f t="shared" si="1"/>
         <v>1808.1318843283225</v>
       </c>
+      <c r="AM35" s="14">
+        <f t="shared" si="1"/>
+        <v>-4678.6624474907294</v>
+      </c>
+      <c r="AN35" s="14">
+        <f t="shared" si="1"/>
+        <v>7361.191866712179</v>
+      </c>
+      <c r="AO35" s="14">
+        <f t="shared" si="1"/>
+        <v>9050.7094574974617</v>
+      </c>
+      <c r="AP35" s="14">
+        <f t="shared" si="1"/>
+        <v>10757.607047656435</v>
+      </c>
+      <c r="AQ35" s="14">
+        <f t="shared" si="1"/>
+        <v>-7339.0219950611936</v>
+      </c>
+      <c r="AR35" s="14">
+        <f t="shared" si="1"/>
+        <v>-4362.9051971435547</v>
+      </c>
+      <c r="AS35" s="14">
+        <f t="shared" si="1"/>
+        <v>-37705.681494973251</v>
+      </c>
     </row>
-    <row r="36" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>21</v>
       </c>
@@ -4885,7 +5539,7 @@
         <v>-155067.73181294976</v>
       </c>
       <c r="D36" s="14">
-        <f t="shared" ref="D36:AL36" si="3">D8-C8</f>
+        <f t="shared" ref="D36:AS36" si="3">D8-C8</f>
         <v>46514.19802570052</v>
       </c>
       <c r="E36" s="14">
@@ -5024,8 +5678,36 @@
         <f t="shared" si="3"/>
         <v>9669.3163340715691</v>
       </c>
+      <c r="AM36" s="14">
+        <f t="shared" si="3"/>
+        <v>-3794.2363494092133</v>
+      </c>
+      <c r="AN36" s="14">
+        <f t="shared" si="3"/>
+        <v>-28045.975958212046</v>
+      </c>
+      <c r="AO36" s="14">
+        <f t="shared" si="3"/>
+        <v>14456.865909302258</v>
+      </c>
+      <c r="AP36" s="14">
+        <f t="shared" si="3"/>
+        <v>9391.1080845437245</v>
+      </c>
+      <c r="AQ36" s="14">
+        <f t="shared" si="3"/>
+        <v>5760.5334200608777</v>
+      </c>
+      <c r="AR36" s="14">
+        <f t="shared" si="3"/>
+        <v>7246.3038071435876</v>
+      </c>
+      <c r="AS36" s="14">
+        <f t="shared" si="3"/>
+        <v>15368.286321973312</v>
+      </c>
     </row>
-    <row r="37" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>2</v>
       </c>
@@ -5035,7 +5717,7 @@
         <v>-107111.0791586999</v>
       </c>
       <c r="D37" s="14">
-        <f t="shared" ref="D37:AL37" si="4">D9-C9</f>
+        <f t="shared" ref="D37:AS37" si="4">D9-C9</f>
         <v>39857.426203499839</v>
       </c>
       <c r="E37" s="14">
@@ -5174,8 +5856,36 @@
         <f t="shared" si="4"/>
         <v>10454.108354399912</v>
       </c>
+      <c r="AM37" s="14">
+        <f t="shared" si="4"/>
+        <v>244.27343319996726</v>
+      </c>
+      <c r="AN37" s="14">
+        <f t="shared" si="4"/>
+        <v>844.65435870003421</v>
+      </c>
+      <c r="AO37" s="14">
+        <f t="shared" si="4"/>
+        <v>-38046.852633700008</v>
+      </c>
+      <c r="AP37" s="14">
+        <f t="shared" si="4"/>
+        <v>8799.37771050015</v>
+      </c>
+      <c r="AQ37" s="14">
+        <f t="shared" si="4"/>
+        <v>4624.8893189999508</v>
+      </c>
+      <c r="AR37" s="14">
+        <f t="shared" si="4"/>
+        <v>7004.3696101000533</v>
+      </c>
+      <c r="AS37" s="14">
+        <f t="shared" si="4"/>
+        <v>15146.677455599769</v>
+      </c>
     </row>
-    <row r="38" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>3</v>
       </c>
@@ -5185,7 +5895,7 @@
         <v>-51069.012459399994</v>
       </c>
       <c r="D38" s="14">
-        <f t="shared" ref="D38:AL38" si="5">D10-C10</f>
+        <f t="shared" ref="D38:AS38" si="5">D10-C10</f>
         <v>8005.8553024999565</v>
       </c>
       <c r="E38" s="14">
@@ -5324,8 +6034,36 @@
         <f t="shared" si="5"/>
         <v>-1184.4430963001214</v>
       </c>
+      <c r="AM38" s="14">
+        <f t="shared" si="5"/>
+        <v>-6482.9173279999522</v>
+      </c>
+      <c r="AN38" s="14">
+        <f t="shared" si="5"/>
+        <v>-26358.486448199954</v>
+      </c>
+      <c r="AO38" s="14">
+        <f t="shared" si="5"/>
+        <v>30125.546524800011</v>
+      </c>
+      <c r="AP38" s="14">
+        <f t="shared" si="5"/>
+        <v>158.72644830006175</v>
+      </c>
+      <c r="AQ38" s="14">
+        <f t="shared" si="5"/>
+        <v>2482.930103099905</v>
+      </c>
+      <c r="AR38" s="14">
+        <f t="shared" si="5"/>
+        <v>470.46105089993216</v>
+      </c>
+      <c r="AS38" s="14">
+        <f t="shared" si="5"/>
+        <v>254.36923079995904</v>
+      </c>
     </row>
-    <row r="39" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>17</v>
       </c>
@@ -5335,7 +6073,7 @@
         <v>-50370.300723999972</v>
       </c>
       <c r="D39" s="14">
-        <f t="shared" ref="D39:AL39" si="6">D11-C11</f>
+        <f t="shared" ref="D39:AS39" si="6">D11-C11</f>
         <v>5074.7103159999824</v>
       </c>
       <c r="E39" s="14">
@@ -5474,8 +6212,36 @@
         <f t="shared" si="6"/>
         <v>104.94539100001566</v>
       </c>
+      <c r="AM39" s="14">
+        <f t="shared" si="6"/>
+        <v>314.83617699996103</v>
+      </c>
+      <c r="AN39" s="14">
+        <f t="shared" si="6"/>
+        <v>104.94538900000043</v>
+      </c>
+      <c r="AO39" s="14">
+        <f t="shared" si="6"/>
+        <v>14370.327649999992</v>
+      </c>
+      <c r="AP39" s="14">
+        <f t="shared" si="6"/>
+        <v>107.60934800002724</v>
+      </c>
+      <c r="AQ39" s="14">
+        <f t="shared" si="6"/>
+        <v>107.6093520000577</v>
+      </c>
+      <c r="AR39" s="14">
+        <f t="shared" si="6"/>
+        <v>322.82804799999576</v>
+      </c>
+      <c r="AS39" s="14">
+        <f t="shared" si="6"/>
+        <v>107.60935099993367</v>
+      </c>
     </row>
-    <row r="40" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>22</v>
       </c>
@@ -5485,7 +6251,7 @@
         <v>19703.07854800002</v>
       </c>
       <c r="D40" s="14">
-        <f t="shared" ref="D40:AL40" si="7">D12-C12</f>
+        <f t="shared" ref="D40:AS40" si="7">D12-C12</f>
         <v>5074.7103159999824</v>
       </c>
       <c r="E40" s="14">
@@ -5624,8 +6390,36 @@
         <f t="shared" si="7"/>
         <v>104.94539100001566</v>
       </c>
+      <c r="AM40" s="14">
+        <f t="shared" si="7"/>
+        <v>314.83617699996103</v>
+      </c>
+      <c r="AN40" s="14">
+        <f t="shared" si="7"/>
+        <v>104.94538900000043</v>
+      </c>
+      <c r="AO40" s="14">
+        <f t="shared" si="7"/>
+        <v>14370.327649999992</v>
+      </c>
+      <c r="AP40" s="14">
+        <f t="shared" si="7"/>
+        <v>107.60934800002724</v>
+      </c>
+      <c r="AQ40" s="14">
+        <f t="shared" si="7"/>
+        <v>107.60935199994128</v>
+      </c>
+      <c r="AR40" s="14">
+        <f t="shared" si="7"/>
+        <v>322.82804799999576</v>
+      </c>
+      <c r="AS40" s="14">
+        <f t="shared" si="7"/>
+        <v>107.60935100005008</v>
+      </c>
     </row>
-    <row r="41" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>23</v>
       </c>
@@ -5635,7 +6429,7 @@
         <v>0</v>
       </c>
       <c r="D41" s="14">
-        <f t="shared" ref="D41:AL41" si="8">D13-C13</f>
+        <f t="shared" ref="D41:AS41" si="8">D13-C13</f>
         <v>0</v>
       </c>
       <c r="E41" s="14">
@@ -5774,8 +6568,36 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
+      <c r="AM41" s="14">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AN41" s="14">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AO41" s="14">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AP41" s="14">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AQ41" s="14">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AR41" s="14">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AS41" s="14">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="42" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>24</v>
       </c>
@@ -5785,7 +6607,7 @@
         <v>-70073.379272000006</v>
       </c>
       <c r="D42" s="14">
-        <f t="shared" ref="D42:AL42" si="9">D14-C14</f>
+        <f t="shared" ref="D42:AS42" si="9">D14-C14</f>
         <v>0</v>
       </c>
       <c r="E42" s="14">
@@ -5924,8 +6746,36 @@
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
+      <c r="AM42" s="14">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="AN42" s="14">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="AO42" s="14">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="AP42" s="14">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="AQ42" s="14">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="AR42" s="14">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="AS42" s="14">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="43" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>25</v>
       </c>
@@ -5935,7 +6785,7 @@
         <v>0</v>
       </c>
       <c r="D43" s="14">
-        <f t="shared" ref="D43:AL43" si="10">D15-C15</f>
+        <f t="shared" ref="D43:AS43" si="10">D15-C15</f>
         <v>0</v>
       </c>
       <c r="E43" s="14">
@@ -6074,8 +6924,36 @@
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
+      <c r="AM43" s="14">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AN43" s="14">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AO43" s="14">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AP43" s="14">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AQ43" s="14">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AR43" s="14">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AS43" s="14">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="44" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>9</v>
       </c>
@@ -6085,7 +6963,7 @@
         <v>0</v>
       </c>
       <c r="D44" s="14">
-        <f t="shared" ref="D44:AL44" si="11">D16-C16</f>
+        <f t="shared" ref="D44:AS44" si="11">D16-C16</f>
         <v>0</v>
       </c>
       <c r="E44" s="14">
@@ -6224,8 +7102,36 @@
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
+      <c r="AM44" s="14">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AN44" s="14">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AO44" s="14">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AP44" s="14">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AQ44" s="14">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AR44" s="14">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="AS44" s="14">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="45" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>10</v>
       </c>
@@ -6235,7 +7141,7 @@
         <v>0</v>
       </c>
       <c r="D45" s="14">
-        <f t="shared" ref="D45:AL45" si="12">-(D17-C17)</f>
+        <f t="shared" ref="D45:AS45" si="12">-(D17-C17)</f>
         <v>0</v>
       </c>
       <c r="E45" s="14">
@@ -6374,8 +7280,36 @@
         <f t="shared" si="12"/>
         <v>3000.4315068000001</v>
       </c>
+      <c r="AM45" s="14">
+        <f t="shared" si="12"/>
+        <v>6950.9996576000012</v>
+      </c>
+      <c r="AN45" s="14">
+        <f t="shared" si="12"/>
+        <v>26503.811643800003</v>
+      </c>
+      <c r="AO45" s="14">
+        <f t="shared" si="12"/>
+        <v>-36455.242808200004</v>
+      </c>
+      <c r="AP45" s="14">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AQ45" s="14">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AR45" s="14">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="AS45" s="14">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="46" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>12</v>
       </c>
@@ -6385,7 +7319,7 @@
         <v>0</v>
       </c>
       <c r="D46" s="14">
-        <f t="shared" ref="D46:AL46" si="13">-(D18-C18)</f>
+        <f t="shared" ref="D46:AS46" si="13">-(D18-C18)</f>
         <v>0</v>
       </c>
       <c r="E46" s="14">
@@ -6524,8 +7458,36 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
+      <c r="AM46" s="14">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="AN46" s="14">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="AO46" s="14">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="AP46" s="14">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="AQ46" s="14">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="AR46" s="14">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="AS46" s="14">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="47" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>18</v>
       </c>
@@ -6535,7 +7497,7 @@
         <v>0</v>
       </c>
       <c r="D47" s="14">
-        <f t="shared" ref="D47:AL47" si="14">-(D19-C19)</f>
+        <f t="shared" ref="D47:AS47" si="14">-(D19-C19)</f>
         <v>0</v>
       </c>
       <c r="E47" s="14">
@@ -6674,8 +7636,36 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
+      <c r="AM47" s="14">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="AN47" s="14">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="AO47" s="14">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="AP47" s="14">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="AQ47" s="14">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="AR47" s="14">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="AS47" s="14">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="48" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>11</v>
       </c>
@@ -6685,7 +7675,7 @@
         <v>0</v>
       </c>
       <c r="D48" s="14">
-        <f t="shared" ref="D48:AL48" si="15">-(D20-C20)</f>
+        <f t="shared" ref="D48:AS48" si="15">-(D20-C20)</f>
         <v>0</v>
       </c>
       <c r="E48" s="14">
@@ -6824,8 +7814,36 @@
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
+      <c r="AM48" s="14">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="AN48" s="14">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="AO48" s="14">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="AP48" s="14">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="AQ48" s="14">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="AR48" s="14">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="AS48" s="14">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="49" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>16</v>
       </c>
@@ -6835,7 +7853,7 @@
         <v>0</v>
       </c>
       <c r="D49" s="14">
-        <f t="shared" ref="D49:AL49" si="16">-(D21-C21)</f>
+        <f t="shared" ref="D49:AS49" si="16">-(D21-C21)</f>
         <v>0</v>
       </c>
       <c r="E49" s="14">
@@ -6974,8 +7992,36 @@
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
+      <c r="AM49" s="14">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="AN49" s="14">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="AO49" s="14">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="AP49" s="14">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="AQ49" s="14">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="AR49" s="14">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="AS49" s="14">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="50" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>20</v>
       </c>
@@ -6985,7 +8031,7 @@
         <v>3112.3598051503068</v>
       </c>
       <c r="D50" s="14">
-        <f t="shared" ref="D50:AL50" si="17">D22-C22</f>
+        <f t="shared" ref="D50:AS50" si="17">D22-C22</f>
         <v>-1349.083480299334</v>
       </c>
       <c r="E50" s="14">
@@ -7124,8 +8170,36 @@
         <f t="shared" si="17"/>
         <v>399.65107597177848</v>
       </c>
+      <c r="AM50" s="14">
+        <f t="shared" si="17"/>
+        <v>2444.4075453908881</v>
+      </c>
+      <c r="AN50" s="14">
+        <f t="shared" si="17"/>
+        <v>-2532.1438687122427</v>
+      </c>
+      <c r="AO50" s="14">
+        <f t="shared" si="17"/>
+        <v>22378.172018202371</v>
+      </c>
+      <c r="AP50" s="14">
+        <f t="shared" si="17"/>
+        <v>433.00392574351281</v>
+      </c>
+      <c r="AQ50" s="14">
+        <f t="shared" si="17"/>
+        <v>-1347.286002038978</v>
+      </c>
+      <c r="AR50" s="14">
+        <f t="shared" si="17"/>
+        <v>-228.52685385639779</v>
+      </c>
+      <c r="AS50" s="14">
+        <f t="shared" si="17"/>
+        <v>-32.760364426416345</v>
+      </c>
     </row>
-    <row r="51" spans="1:38" s="21" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:45" s="21" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A51" s="19" t="s">
         <v>4</v>
       </c>
@@ -7135,7 +8209,7 @@
         <v>-165677.11378010013</v>
       </c>
       <c r="D51" s="22">
-        <f t="shared" ref="D51:AL51" si="18">D23-C23</f>
+        <f t="shared" ref="D51:AS51" si="18">D23-C23</f>
         <v>-30155.64123570011</v>
       </c>
       <c r="E51" s="22">
@@ -7274,8 +8348,36 @@
         <f t="shared" si="18"/>
         <v>11477.448218399892</v>
       </c>
+      <c r="AM51" s="22">
+        <f t="shared" si="18"/>
+        <v>-8472.8987968999427</v>
+      </c>
+      <c r="AN51" s="22">
+        <f t="shared" si="18"/>
+        <v>-20684.784091499867</v>
+      </c>
+      <c r="AO51" s="22">
+        <f t="shared" si="18"/>
+        <v>23507.57536679972</v>
+      </c>
+      <c r="AP51" s="22">
+        <f t="shared" si="18"/>
+        <v>20148.715132200159</v>
+      </c>
+      <c r="AQ51" s="22">
+        <f t="shared" si="18"/>
+        <v>-1578.4885750003159</v>
+      </c>
+      <c r="AR51" s="22">
+        <f t="shared" si="18"/>
+        <v>2883.3986100000329</v>
+      </c>
+      <c r="AS51" s="22">
+        <f t="shared" si="18"/>
+        <v>-22337.395172999939</v>
+      </c>
     </row>
-    <row r="52" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>5</v>
       </c>
@@ -7285,7 +8387,7 @@
         <v>-59383.53690019995</v>
       </c>
       <c r="D52" s="14">
-        <f t="shared" ref="D52:AL52" si="19">D24-C24</f>
+        <f t="shared" ref="D52:AS52" si="19">D24-C24</f>
         <v>-6249.2710569000337</v>
       </c>
       <c r="E52" s="14">
@@ -7424,8 +8526,36 @@
         <f t="shared" si="19"/>
         <v>4706.6294100000523</v>
       </c>
+      <c r="AM52" s="14">
+        <f t="shared" si="19"/>
+        <v>3246.2570491998922</v>
+      </c>
+      <c r="AN52" s="14">
+        <f t="shared" si="19"/>
+        <v>562.77886570000555</v>
+      </c>
+      <c r="AO52" s="14">
+        <f t="shared" si="19"/>
+        <v>-2175.8941999999806</v>
+      </c>
+      <c r="AP52" s="14">
+        <f t="shared" si="19"/>
+        <v>-10.439869599998929</v>
+      </c>
+      <c r="AQ52" s="14">
+        <f t="shared" si="19"/>
+        <v>3615.7531500000041</v>
+      </c>
+      <c r="AR52" s="14">
+        <f t="shared" si="19"/>
+        <v>-778.18861909990665</v>
+      </c>
+      <c r="AS52" s="14">
+        <f t="shared" si="19"/>
+        <v>-1835.8083690000931</v>
+      </c>
     </row>
-    <row r="53" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>14</v>
       </c>
@@ -7435,7 +8565,7 @@
         <v>-86833.387378500018</v>
       </c>
       <c r="D53" s="14">
-        <f t="shared" ref="D53:AL53" si="20">D25-C25</f>
+        <f t="shared" ref="D53:AS53" si="20">D25-C25</f>
         <v>-6423.7477292000549</v>
       </c>
       <c r="E53" s="14">
@@ -7574,8 +8704,36 @@
         <f t="shared" si="20"/>
         <v>6489.4581387999933</v>
       </c>
+      <c r="AM53" s="14">
+        <f t="shared" si="20"/>
+        <v>-5416.9468660999555</v>
+      </c>
+      <c r="AN53" s="14">
+        <f t="shared" si="20"/>
+        <v>-25232.576580100053</v>
+      </c>
+      <c r="AO53" s="14">
+        <f t="shared" si="20"/>
+        <v>18574.222176900017</v>
+      </c>
+      <c r="AP53" s="14">
+        <f t="shared" si="20"/>
+        <v>10913.130180599983</v>
+      </c>
+      <c r="AQ53" s="14">
+        <f t="shared" si="20"/>
+        <v>-7677.0521187999984</v>
+      </c>
+      <c r="AR53" s="14">
+        <f t="shared" si="20"/>
+        <v>-37.993324899987783</v>
+      </c>
+      <c r="AS53" s="14">
+        <f t="shared" si="20"/>
+        <v>-7274.3405135000357</v>
+      </c>
     </row>
-    <row r="54" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>13</v>
       </c>
@@ -7585,7 +8743,7 @@
         <v>8808.5551820000401</v>
       </c>
       <c r="D54" s="14">
-        <f t="shared" ref="D54:AL54" si="21">D26-C26</f>
+        <f t="shared" ref="D54:AS54" si="21">D26-C26</f>
         <v>-19555.200326499995</v>
       </c>
       <c r="E54" s="14">
@@ -7724,8 +8882,36 @@
         <f t="shared" si="21"/>
         <v>-638.67184900003485</v>
       </c>
+      <c r="AM54" s="14">
+        <f t="shared" si="21"/>
+        <v>-2561.8088797000237</v>
+      </c>
+      <c r="AN54" s="14">
+        <f t="shared" si="21"/>
+        <v>2721.0981846000068</v>
+      </c>
+      <c r="AO54" s="14">
+        <f t="shared" si="21"/>
+        <v>6967.4373368999804</v>
+      </c>
+      <c r="AP54" s="14">
+        <f t="shared" si="21"/>
+        <v>7100.7980852000182</v>
+      </c>
+      <c r="AQ54" s="14">
+        <f t="shared" si="21"/>
+        <v>6305.7759056999348</v>
+      </c>
+      <c r="AR54" s="14">
+        <f t="shared" si="21"/>
+        <v>-3091.3594907999504</v>
+      </c>
+      <c r="AS54" s="14">
+        <f t="shared" si="21"/>
+        <v>-8778.1233742000186</v>
+      </c>
     </row>
-    <row r="55" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
         <v>29</v>
       </c>
@@ -7766,8 +8952,15 @@
       <c r="AJ55" s="14"/>
       <c r="AK55" s="14"/>
       <c r="AL55" s="14"/>
+      <c r="AM55" s="14"/>
+      <c r="AN55" s="14"/>
+      <c r="AO55" s="14"/>
+      <c r="AP55" s="14"/>
+      <c r="AQ55" s="14"/>
+      <c r="AR55" s="14"/>
+      <c r="AS55" s="14"/>
     </row>
-    <row r="56" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>30</v>
       </c>
@@ -7808,8 +9001,15 @@
       <c r="AJ56" s="14"/>
       <c r="AK56" s="14"/>
       <c r="AL56" s="14"/>
+      <c r="AM56" s="14"/>
+      <c r="AN56" s="14"/>
+      <c r="AO56" s="14"/>
+      <c r="AP56" s="14"/>
+      <c r="AQ56" s="14"/>
+      <c r="AR56" s="14"/>
+      <c r="AS56" s="14"/>
     </row>
-    <row r="57" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>6</v>
       </c>
@@ -7819,7 +9019,7 @@
         <v>-28268.744683400204</v>
       </c>
       <c r="D57" s="14">
-        <f t="shared" ref="D57:AL57" si="22">D29-C29</f>
+        <f t="shared" ref="D57:AS57" si="22">D29-C29</f>
         <v>2072.5778768999735</v>
       </c>
       <c r="E57" s="14">
@@ -7958,8 +9158,36 @@
         <f t="shared" si="22"/>
         <v>919.94567009988168</v>
       </c>
+      <c r="AM57" s="14">
+        <f t="shared" si="22"/>
+        <v>-3476.2992903998565</v>
+      </c>
+      <c r="AN57" s="14">
+        <f t="shared" si="22"/>
+        <v>1263.8108886001737</v>
+      </c>
+      <c r="AO57" s="14">
+        <f t="shared" si="22"/>
+        <v>141.31801909970272</v>
+      </c>
+      <c r="AP57" s="14">
+        <f t="shared" si="22"/>
+        <v>2144.9775094001579</v>
+      </c>
+      <c r="AQ57" s="14">
+        <f t="shared" si="22"/>
+        <v>-3823.4083202002566</v>
+      </c>
+      <c r="AR57" s="14">
+        <f t="shared" si="22"/>
+        <v>6790.9422086998784</v>
+      </c>
+      <c r="AS57" s="14">
+        <f t="shared" si="22"/>
+        <v>-4448.7984819997928</v>
+      </c>
     </row>
-    <row r="58" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
         <v>7</v>
       </c>
@@ -7969,7 +9197,7 @@
         <v>-29524.726904799994</v>
       </c>
       <c r="D58" s="14">
-        <f t="shared" ref="D58:AL58" si="23">D30-C30</f>
+        <f t="shared" ref="D58:AS58" si="23">D30-C30</f>
         <v>2421.9176890999952</v>
       </c>
       <c r="E58" s="14">
@@ -8108,8 +9336,36 @@
         <f t="shared" si="23"/>
         <v>15.932580700000472</v>
       </c>
+      <c r="AM58" s="14">
+        <f t="shared" si="23"/>
+        <v>-2369.4851126000012</v>
+      </c>
+      <c r="AN58" s="14">
+        <f t="shared" si="23"/>
+        <v>433.73621880000064</v>
+      </c>
+      <c r="AO58" s="14">
+        <f t="shared" si="23"/>
+        <v>128.36553219999951</v>
+      </c>
+      <c r="AP58" s="14">
+        <f t="shared" si="23"/>
+        <v>-11.039705199998934</v>
+      </c>
+      <c r="AQ58" s="14">
+        <f t="shared" si="23"/>
+        <v>-642.68189070000062</v>
+      </c>
+      <c r="AR58" s="14">
+        <f t="shared" si="23"/>
+        <v>1976.5398723999997</v>
+      </c>
+      <c r="AS58" s="14">
+        <f t="shared" si="23"/>
+        <v>4.9778629000011279</v>
+      </c>
     </row>
-    <row r="59" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>8</v>
       </c>
@@ -8119,7 +9375,7 @@
         <v>1255.9822214000003</v>
       </c>
       <c r="D59" s="14">
-        <f t="shared" ref="D59:AL59" si="24">D31-C31</f>
+        <f t="shared" ref="D59:AS59" si="24">D31-C31</f>
         <v>-349.33981220000078</v>
       </c>
       <c r="E59" s="14">
@@ -8258,26 +9514,54 @@
         <f t="shared" si="24"/>
         <v>904.01308940000035</v>
       </c>
+      <c r="AM59" s="14">
+        <f t="shared" si="24"/>
+        <v>-1106.8141777999995</v>
+      </c>
+      <c r="AN59" s="14">
+        <f t="shared" si="24"/>
+        <v>830.07466979999981</v>
+      </c>
+      <c r="AO59" s="14">
+        <f t="shared" si="24"/>
+        <v>12.952486899999712</v>
+      </c>
+      <c r="AP59" s="14">
+        <f t="shared" si="24"/>
+        <v>2156.0172146000004</v>
+      </c>
+      <c r="AQ59" s="14">
+        <f t="shared" si="24"/>
+        <v>-3180.7264295000004</v>
+      </c>
+      <c r="AR59" s="14">
+        <f t="shared" si="24"/>
+        <v>4814.4023362999997</v>
+      </c>
+      <c r="AS59" s="14">
+        <f t="shared" si="24"/>
+        <v>-4453.7763448999995</v>
+      </c>
     </row>
-    <row r="60" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A60" s="4"/>
     </row>
-    <row r="61" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A61" s="17"/>
     </row>
-    <row r="62" spans="1:38" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:45" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="25" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="63" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A63" s="26" t="s">
         <v>35</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A63" r:id="rId1"/>
+    <hyperlink ref="A63" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
@@ -8414,13 +9698,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{60C41967-BBAB-4701-A650-265D07F6153B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADEA22CB-C5D5-4882-95EC-EBD34BE86ADC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75DFB10F-E8DD-4823-A2B4-94444691B453}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B96C55F6-7D13-415E-B942-8AD48DFD2681}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38584A2C-BF64-4CB1-A00A-25B3B164AD78}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{789900CD-9F06-4FA7-9113-C6DA70872B72}"/>
 </file>
</xml_diff>